<commit_message>
update full pipeline code
</commit_message>
<xml_diff>
--- a/robustness/data/_robustness/all_claims.xlsx
+++ b/robustness/data/_robustness/all_claims.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\mason\mygpu\llm-robustness\llm-benchmarking-robustness\robustness\data\_robustness\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A59B6F5E-2DC5-409B-955C-0D0D45F54FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{984C0B7C-3B68-43D4-8A5F-966BFCAC38C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-6705" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3833,7 +3833,7 @@
     <t>osf.io/deyax</t>
   </si>
   <si>
-    <t>Powell_CompPolitStu_2009_0PZl</t>
+    <t>Bingham Powell_CompPolitStu_2009_0PZl</t>
   </si>
 </sst>
 </file>

</xml_diff>